<commit_message>
fix: remove seeded passwords and separate user activation
</commit_message>
<xml_diff>
--- a/database/seed/TAQADDUM_import_ready.xlsx
+++ b/database/seed/TAQADDUM_import_ready.xlsx
@@ -424,171 +424,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>full_name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>password</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>role_code</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>direction@taqaddum.dz</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Direction CNED</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Taqaddum2026!</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CNED_DIRECTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pmo@taqaddum.dz</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CNED / PMO</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Taqaddum2026!</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CNED_PMO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>mo@taqaddum.dz</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Maître d'ouvrage</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Taqaddum2026!</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>bet@taqaddum.dz</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bureau d'études</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Taqaddum2026!</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>BET</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>entreprise@taqaddum.dz</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Contractant</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Taqaddum2026!</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CONTRACTOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>finance@taqaddum.dz</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Contrôleur budgétaire</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Taqaddum2026!</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>FINANCE</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
+    <ns0:pageSetUpPr/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:D7"/>
+  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>email</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>full_name</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>password</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>role_code</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>direction@taqaddum.dz</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Direction CNED</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" t="inlineStr"/>
+      <ns0:c r="D2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CNED_DIRECTION</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>pmo@taqaddum.dz</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CNED / PMO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" t="inlineStr"/>
+      <ns0:c r="D3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CNED_PMO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mo@taqaddum.dz</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Maître d'ouvrage</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" t="inlineStr"/>
+      <ns0:c r="D4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>bet@taqaddum.dz</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Bureau d'études</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" t="inlineStr"/>
+      <ns0:c r="D5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>BET</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>entreprise@taqaddum.dz</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contractant</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" t="inlineStr"/>
+      <ns0:c r="D6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CONTRACTOR</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>finance@taqaddum.dz</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contrôleur budgétaire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" t="inlineStr"/>
+      <ns0:c r="D7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FINANCE</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>